<commit_message>
ran one flatblock optimization run
</commit_message>
<xml_diff>
--- a/heat_demand/pulp_paper_heat_demand_corrected.xlsx
+++ b/heat_demand/pulp_paper_heat_demand_corrected.xlsx
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="6">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>1.5</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="10">

</xml_diff>